<commit_message>
Renommage entete FHIR f79df3386ccbc740f8fe282ca9d6f9d3b3910aec
</commit_message>
<xml_diff>
--- a/renommage-entete-FHIR/ig/StructureDefinition-fr-bundle-document.xlsx
+++ b/renommage-entete-FHIR/ig/StructureDefinition-fr-bundle-document.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-10-21T21:35:58+00:00</t>
+    <t>2025-10-21T22:51:41+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -576,7 +576,7 @@
     <t>7</t>
   </si>
   <si>
-    <t>Ressource Entry dans le FrBundleDocument</t>
+    <t>Ressource Entry dans le FRBundleDocument</t>
   </si>
   <si>
     <t>Une ressource Entry incluse dans le bundle de ressources du document</t>

</xml_diff>